<commit_message>
Auto update ETF comparison: Fri Jul 24 10:39:36 UTC 2026
</commit_message>
<xml_diff>
--- a/data/00982A/20260724.xlsx
+++ b/data/00982A/20260724.xlsx
@@ -385,7 +385,7 @@
         <v>基金淨資產價值(元)</v>
       </c>
       <c r="B1" t="str">
-        <v>TWD 50,332,910,185</v>
+        <v>TWD 48,139,688,230</v>
       </c>
     </row>
     <row r="2">
@@ -393,7 +393,7 @@
         <v>每受益權單位淨資產價值(元)-台幣交易</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD 22.85</v>
+        <v>TWD 21.86</v>
       </c>
     </row>
     <row r="3">
@@ -413,7 +413,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,7 +437,7 @@
         <v>台積電</v>
       </c>
       <c r="C2" t="str">
-        <v>9.4%</v>
+        <v>9.6%</v>
       </c>
       <c r="D2" t="str">
         <v>1,967,000</v>
@@ -451,7 +451,7 @@
         <v>聖暉*</v>
       </c>
       <c r="C3" t="str">
-        <v>8.96%</v>
+        <v>8.78%</v>
       </c>
       <c r="D3" t="str">
         <v>3,775,000</v>
@@ -465,7 +465,7 @@
         <v>聯發科</v>
       </c>
       <c r="C4" t="str">
-        <v>6.69%</v>
+        <v>6.77%</v>
       </c>
       <c r="D4" t="str">
         <v>869,000</v>
@@ -479,80 +479,80 @@
         <v>亞翔</v>
       </c>
       <c r="C5" t="str">
-        <v>5.28%</v>
+        <v>5.62%</v>
       </c>
       <c r="D5" t="str">
-        <v>3,099,000</v>
+        <v>3,219,000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>6223</v>
+        <v>2345</v>
       </c>
       <c r="B6" t="str">
-        <v>旺矽</v>
+        <v>智邦</v>
       </c>
       <c r="C6" t="str">
-        <v>3.81%</v>
+        <v>3.74%</v>
       </c>
       <c r="D6" t="str">
-        <v>307,000</v>
+        <v>812,000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2345</v>
+        <v>6223</v>
       </c>
       <c r="B7" t="str">
-        <v>智邦</v>
+        <v>旺矽</v>
       </c>
       <c r="C7" t="str">
-        <v>3.75%</v>
+        <v>3.64%</v>
       </c>
       <c r="D7" t="str">
-        <v>812,000</v>
+        <v>307,000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2360</v>
+        <v>6669</v>
       </c>
       <c r="B8" t="str">
-        <v>致茂</v>
+        <v>緯穎</v>
       </c>
       <c r="C8" t="str">
-        <v>3.58%</v>
+        <v>3.62%</v>
       </c>
       <c r="D8" t="str">
-        <v>837,000</v>
+        <v>304,000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2383</v>
+        <v>2360</v>
       </c>
       <c r="B9" t="str">
-        <v>台光電</v>
+        <v>致茂</v>
       </c>
       <c r="C9" t="str">
-        <v>3.36%</v>
+        <v>3.62%</v>
       </c>
       <c r="D9" t="str">
-        <v>332,000</v>
+        <v>837,000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>6669</v>
+        <v>2383</v>
       </c>
       <c r="B10" t="str">
-        <v>緯穎</v>
+        <v>台光電</v>
       </c>
       <c r="C10" t="str">
-        <v>3.3%</v>
+        <v>3.28%</v>
       </c>
       <c r="D10" t="str">
-        <v>304,000</v>
+        <v>332,000</v>
       </c>
     </row>
     <row r="11">
@@ -563,7 +563,7 @@
         <v>臻鼎-KY</v>
       </c>
       <c r="C11" t="str">
-        <v>3.19%</v>
+        <v>3.18%</v>
       </c>
       <c r="D11" t="str">
         <v>3,178,000</v>
@@ -577,7 +577,7 @@
         <v>穩懋</v>
       </c>
       <c r="C12" t="str">
-        <v>3.06%</v>
+        <v>3%</v>
       </c>
       <c r="D12" t="str">
         <v>4,226,000</v>
@@ -591,7 +591,7 @@
         <v>川湖</v>
       </c>
       <c r="C13" t="str">
-        <v>3.01%</v>
+        <v>2.97%</v>
       </c>
       <c r="D13" t="str">
         <v>185,000</v>
@@ -599,30 +599,30 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>3491</v>
+        <v>6488</v>
       </c>
       <c r="B14" t="str">
-        <v>昇達科</v>
+        <v>環球晶</v>
       </c>
       <c r="C14" t="str">
-        <v>2.55%</v>
+        <v>2.45%</v>
       </c>
       <c r="D14" t="str">
-        <v>988,000</v>
+        <v>1,146,000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>6488</v>
+        <v>3491</v>
       </c>
       <c r="B15" t="str">
-        <v>環球晶</v>
+        <v>昇達科</v>
       </c>
       <c r="C15" t="str">
-        <v>2.55%</v>
+        <v>2.44%</v>
       </c>
       <c r="D15" t="str">
-        <v>1,146,000</v>
+        <v>988,000</v>
       </c>
     </row>
     <row r="16">
@@ -633,7 +633,7 @@
         <v>聯電</v>
       </c>
       <c r="C16" t="str">
-        <v>2.49%</v>
+        <v>2.41%</v>
       </c>
       <c r="D16" t="str">
         <v>9,065,000</v>
@@ -647,7 +647,7 @@
         <v>矽格</v>
       </c>
       <c r="C17" t="str">
-        <v>2.12%</v>
+        <v>2.13%</v>
       </c>
       <c r="D17" t="str">
         <v>4,717,000</v>
@@ -661,7 +661,7 @@
         <v>欣銓</v>
       </c>
       <c r="C18" t="str">
-        <v>2.07%</v>
+        <v>2.08%</v>
       </c>
       <c r="D18" t="str">
         <v>4,780,000</v>
@@ -675,7 +675,7 @@
         <v>愛普*</v>
       </c>
       <c r="C19" t="str">
-        <v>2.03%</v>
+        <v>2.01%</v>
       </c>
       <c r="D19" t="str">
         <v>1,130,000</v>
@@ -683,30 +683,30 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>3008</v>
+        <v>3017</v>
       </c>
       <c r="B20" t="str">
-        <v>大立光</v>
+        <v>奇鋐</v>
       </c>
       <c r="C20" t="str">
-        <v>2%</v>
+        <v>2.01%</v>
       </c>
       <c r="D20" t="str">
-        <v>243,000</v>
+        <v>407,000</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>3017</v>
+        <v>3008</v>
       </c>
       <c r="B21" t="str">
-        <v>奇鋐</v>
+        <v>大立光</v>
       </c>
       <c r="C21" t="str">
-        <v>1.97%</v>
+        <v>1.98%</v>
       </c>
       <c r="D21" t="str">
-        <v>407,000</v>
+        <v>243,000</v>
       </c>
     </row>
     <row r="22">
@@ -717,7 +717,7 @@
         <v>微星</v>
       </c>
       <c r="C22" t="str">
-        <v>1.73%</v>
+        <v>1.74%</v>
       </c>
       <c r="D22" t="str">
         <v>5,722,000</v>
@@ -731,7 +731,7 @@
         <v>辛耘</v>
       </c>
       <c r="C23" t="str">
-        <v>1.7%</v>
+        <v>1.68%</v>
       </c>
       <c r="D23" t="str">
         <v>1,130,000</v>
@@ -753,58 +753,58 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>3702</v>
+        <v>8016</v>
       </c>
       <c r="B25" t="str">
-        <v>大聯大</v>
+        <v>矽創</v>
       </c>
       <c r="C25" t="str">
-        <v>1.34%</v>
+        <v>1.36%</v>
       </c>
       <c r="D25" t="str">
-        <v>5,565,000</v>
+        <v>2,228,000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>8016</v>
+        <v>3702</v>
       </c>
       <c r="B26" t="str">
-        <v>矽創</v>
+        <v>大聯大</v>
       </c>
       <c r="C26" t="str">
-        <v>1.32%</v>
+        <v>1.36%</v>
       </c>
       <c r="D26" t="str">
-        <v>2,228,000</v>
+        <v>5,565,000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2472</v>
+        <v>3711</v>
       </c>
       <c r="B27" t="str">
-        <v>立隆電</v>
+        <v>日月光投控</v>
       </c>
       <c r="C27" t="str">
-        <v>1.31%</v>
+        <v>1.29%</v>
       </c>
       <c r="D27" t="str">
-        <v>2,383,000</v>
+        <v>1,011,000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>3711</v>
+        <v>2472</v>
       </c>
       <c r="B28" t="str">
-        <v>日月光投控</v>
+        <v>立隆電</v>
       </c>
       <c r="C28" t="str">
-        <v>1.3%</v>
+        <v>1.28%</v>
       </c>
       <c r="D28" t="str">
-        <v>1,011,000</v>
+        <v>2,383,000</v>
       </c>
     </row>
     <row r="29">
@@ -815,7 +815,7 @@
         <v>鴻勁</v>
       </c>
       <c r="C29" t="str">
-        <v>1.19%</v>
+        <v>1.17%</v>
       </c>
       <c r="D29" t="str">
         <v>93,000</v>
@@ -829,7 +829,7 @@
         <v>台燿</v>
       </c>
       <c r="C30" t="str">
-        <v>1.19%</v>
+        <v>1.16%</v>
       </c>
       <c r="D30" t="str">
         <v>447,000</v>
@@ -843,7 +843,7 @@
         <v>國巨*</v>
       </c>
       <c r="C31" t="str">
-        <v>1.17%</v>
+        <v>1.13%</v>
       </c>
       <c r="D31" t="str">
         <v>844,000</v>
@@ -857,7 +857,7 @@
         <v>楠梓電</v>
       </c>
       <c r="C32" t="str">
-        <v>1.13%</v>
+        <v>1.12%</v>
       </c>
       <c r="D32" t="str">
         <v>3,451,000</v>
@@ -865,30 +865,30 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>1785</v>
+        <v>3036</v>
       </c>
       <c r="B33" t="str">
-        <v>光洋科</v>
+        <v>文曄</v>
       </c>
       <c r="C33" t="str">
-        <v>0.97%</v>
+        <v>1%</v>
       </c>
       <c r="D33" t="str">
-        <v>4,461,000</v>
+        <v>2,336,000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>3036</v>
+        <v>1785</v>
       </c>
       <c r="B34" t="str">
-        <v>文曄</v>
+        <v>光洋科</v>
       </c>
       <c r="C34" t="str">
-        <v>0.96%</v>
+        <v>0.98%</v>
       </c>
       <c r="D34" t="str">
-        <v>2,336,000</v>
+        <v>4,461,000</v>
       </c>
     </row>
     <row r="35">
@@ -913,7 +913,7 @@
         <v>高力</v>
       </c>
       <c r="C36" t="str">
-        <v>0.82%</v>
+        <v>0.8%</v>
       </c>
       <c r="D36" t="str">
         <v>382,000</v>
@@ -927,7 +927,7 @@
         <v>技嘉</v>
       </c>
       <c r="C37" t="str">
-        <v>0.75%</v>
+        <v>0.78%</v>
       </c>
       <c r="D37" t="str">
         <v>1,065,000</v>
@@ -955,7 +955,7 @@
         <v>順德</v>
       </c>
       <c r="C39" t="str">
-        <v>0.56%</v>
+        <v>0.58%</v>
       </c>
       <c r="D39" t="str">
         <v>1,729,000</v>
@@ -969,7 +969,7 @@
         <v>力旺</v>
       </c>
       <c r="C40" t="str">
-        <v>0.46%</v>
+        <v>0.48%</v>
       </c>
       <c r="D40" t="str">
         <v>93,000</v>
@@ -977,58 +977,58 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>6147</v>
+        <v>6239</v>
       </c>
       <c r="B41" t="str">
-        <v>頎邦</v>
+        <v>力成</v>
       </c>
       <c r="C41" t="str">
-        <v>0.42%</v>
+        <v>0.41%</v>
       </c>
       <c r="D41" t="str">
-        <v>1,209,000</v>
+        <v>700,000</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>6239</v>
+        <v>6147</v>
       </c>
       <c r="B42" t="str">
-        <v>力成</v>
+        <v>頎邦</v>
       </c>
       <c r="C42" t="str">
-        <v>0.41%</v>
+        <v>0.4%</v>
       </c>
       <c r="D42" t="str">
-        <v>700,000</v>
+        <v>1,209,000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2885</v>
+        <v>2451</v>
       </c>
       <c r="B43" t="str">
-        <v>元大金</v>
+        <v>創見</v>
       </c>
       <c r="C43" t="str">
-        <v>0.27%</v>
+        <v>0.29%</v>
       </c>
       <c r="D43" t="str">
-        <v>2,128,420</v>
+        <v>530,000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2451</v>
+        <v>2885</v>
       </c>
       <c r="B44" t="str">
-        <v>創見</v>
+        <v>元大金</v>
       </c>
       <c r="C44" t="str">
-        <v>0.26%</v>
+        <v>0.28%</v>
       </c>
       <c r="D44" t="str">
-        <v>530,000</v>
+        <v>2,128,420</v>
       </c>
     </row>
     <row r="45">
@@ -1039,7 +1039,7 @@
         <v>萬潤</v>
       </c>
       <c r="C45" t="str">
-        <v>0.19%</v>
+        <v>0.18%</v>
       </c>
       <c r="D45" t="str">
         <v>91,000</v>
@@ -1047,147 +1047,161 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>6177</v>
+        <v>3231</v>
       </c>
       <c r="B46" t="str">
-        <v>達麗</v>
+        <v>緯創</v>
       </c>
       <c r="C46" t="str">
-        <v>0.02%</v>
+        <v>0.04%</v>
       </c>
       <c r="D46" t="str">
-        <v>194,350</v>
+        <v>100,000</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>3443</v>
+        <v>6177</v>
       </c>
       <c r="B47" t="str">
-        <v>創意</v>
+        <v>達麗</v>
       </c>
       <c r="C47" t="str">
-        <v>0.01%</v>
+        <v>0.02%</v>
       </c>
       <c r="D47" t="str">
-        <v>1,000</v>
+        <v>194,350</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>6831</v>
+        <v>3443</v>
       </c>
       <c r="B48" t="str">
-        <v>邁科</v>
+        <v>創意</v>
       </c>
       <c r="C48" t="str">
         <v>0.01%</v>
       </c>
       <c r="D48" t="str">
-        <v>4,000</v>
+        <v>1,000</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>8046</v>
+        <v>6831</v>
       </c>
       <c r="B49" t="str">
-        <v>南電</v>
+        <v>邁科</v>
       </c>
       <c r="C49" t="str">
-        <v>0%</v>
+        <v>0.01%</v>
       </c>
       <c r="D49" t="str">
-        <v>1,000</v>
+        <v>4,000</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>4441</v>
+        <v>8046</v>
       </c>
       <c r="B50" t="str">
-        <v>振大環球</v>
+        <v>南電</v>
       </c>
       <c r="C50" t="str">
         <v>0%</v>
       </c>
       <c r="D50" t="str">
-        <v>4,000</v>
+        <v>1,000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>1519</v>
+        <v>4441</v>
       </c>
       <c r="B51" t="str">
-        <v>華城</v>
+        <v>振大環球</v>
       </c>
       <c r="C51" t="str">
         <v>0%</v>
       </c>
       <c r="D51" t="str">
-        <v>600</v>
+        <v>4,000</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>8358</v>
+        <v>1519</v>
       </c>
       <c r="B52" t="str">
-        <v>金居</v>
+        <v>華城</v>
       </c>
       <c r="C52" t="str">
         <v>0%</v>
       </c>
       <c r="D52" t="str">
-        <v>1,000</v>
+        <v>600</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>3706</v>
+        <v>8358</v>
       </c>
       <c r="B53" t="str">
-        <v>神達</v>
+        <v>金居</v>
       </c>
       <c r="C53" t="str">
         <v>0%</v>
       </c>
       <c r="D53" t="str">
-        <v>1,400</v>
+        <v>1,000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2886</v>
+        <v>3706</v>
       </c>
       <c r="B54" t="str">
-        <v>兆豐金</v>
+        <v>神達</v>
       </c>
       <c r="C54" t="str">
         <v>0%</v>
       </c>
       <c r="D54" t="str">
-        <v>1,000</v>
+        <v>1,400</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2881</v>
+        <v>2886</v>
       </c>
       <c r="B55" t="str">
-        <v>富邦金</v>
+        <v>兆豐金</v>
       </c>
       <c r="C55" t="str">
         <v>0%</v>
       </c>
       <c r="D55" t="str">
+        <v>1,000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2881</v>
+      </c>
+      <c r="B56" t="str">
+        <v>富邦金</v>
+      </c>
+      <c r="C56" t="str">
+        <v>0%</v>
+      </c>
+      <c r="D56" t="str">
         <v>250</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D56"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1252,7 +1266,7 @@
         <v>應收付證券款</v>
       </c>
       <c r="B2" t="str">
-        <v>TWD -276,852,897.00</v>
+        <v>TWD 72,117,046.00</v>
       </c>
     </row>
     <row r="3">
@@ -1268,7 +1282,7 @@
         <v>現金</v>
       </c>
       <c r="B4" t="str">
-        <v>TWD 1,136,735,680.00</v>
+        <v>TWD 759,741,266.00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>